<commit_message>
Trim the academic corpus and adopt Mini Forest column names
Removes four columns from Paper_analysis (32 -> 28): the verbatim 'Results'
and 'Notes' free-text columns, an empty column, and an unlabelled trailing
column holding six site-location links.

Renames three column headings to Mini Forest wording and updates the lookups
in every script that reads them:
  Empirical data on Miyawaki forest?  ->  Empirical data on Mini Forest?
  Miyawaki forest age (years)         ->  Mini Forest age (years)
  Replicated Miyawaki forests?        ->  Replicated Mini Forests?

Eight free-text Measurements cells reworded. Paper titles, the author name
Miyawaki, and the Boolean search string on README_filter are unchanged --
those are the published record.

'Results' was carried only into the QA audit CSV, never into Figure 2 or the
Table S1 document, so that column is dropped from both scripts. Figures 1, 2
and S1 are unchanged: the funnel is still 108/67/33/8/0/0.
</commit_message>
<xml_diff>
--- a/data/Mini_Forest_academic_corpus.xlsx
+++ b/data/Mini_Forest_academic_corpus.xlsx
@@ -695,6 +695,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -825,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="10.83203125" customWidth="1" style="24" min="20" max="21"/>
@@ -906,7 +907,7 @@
       </c>
       <c r="O1" s="3" t="inlineStr">
         <is>
-          <t>Empirical data on Miyawaki forest?</t>
+          <t>Empirical data on Mini Forest?</t>
         </is>
       </c>
       <c r="P1" s="3" t="inlineStr">
@@ -931,7 +932,7 @@
       </c>
       <c r="T1" s="22" t="inlineStr">
         <is>
-          <t>Miyawaki forest age (years)</t>
+          <t>Mini Forest age (years)</t>
         </is>
       </c>
       <c r="U1" s="22" t="inlineStr">
@@ -956,7 +957,7 @@
       </c>
       <c r="Y1" s="4" t="inlineStr">
         <is>
-          <t>Replicated Miyawaki forests?</t>
+          <t>Replicated Mini Forests?</t>
         </is>
       </c>
       <c r="Z1" s="4" t="inlineStr">
@@ -972,17 +973,6 @@
       <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>Statistical tests of claim against other types of urban tree planting?</t>
-        </is>
-      </c>
-      <c r="AC1" s="4" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="AD1" s="4" t="n"/>
-      <c r="AE1" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1123,11 +1113,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Respondents think urban green spaces contribute to feelings of well-being and provide biodiversity support and that more complex spaces contribute more cultural ecosystem services. Tiny forests were percieved as best at providing provisioning and environment-regulating ecosystem services, lawns the least beneficial. Respondents expressed a desire to be directly involved in urban green space design, construction, and maintenance, mostly for increased social interaction.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1261,12 +1246,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC3" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Academics were least engaged or aware of costs associated with Mini Forests. Volunteer communities were most engaged and aware of costs. Public sector professionals were significantly more willing to pay for Mini forests. PhD level, middle-aged, and male professionals were less in favor of using Mini Forests. Those more familiar / involved believing MF is more suitable for the urban (P &lt; 0.001) and less so for the rural environment. Parks/public gardens, river corridors, and educational sites were identified as the three most suitable locations for Mini Forests.When informed about climate change, respondents were more likely to agree with the use of mixed hative and non-native species in MF. </t>
-        </is>
-      </c>
-      <c r="AD3" s="9" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -1401,16 +1380,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>Significant variation among plots in soil physicochemical properties, soil chemistry, bacterial and fungal CFU counts, and soil enzyme activities.</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>There are replicate Miyawaki forest plots, but no replicated control or "traditional method" plots. This is the extent of the treatment description: "Some of the woodlands were reformed by traditional methods and Miyawaki Method and untransformed woodlands were used as control plots". We do not know what the "traditional method" is, except that there was planting there at 0.16 plants per m2 vs. 2-4 plants per m2 for Miyawaki forests. On the edge of Hong Kong, Guangdong Province: https://maps.app.goo.gl/o6YQEHwZu7JZYjEn8</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1542,16 +1511,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Estimated carbon sequestration rate of Miyawaki Forest is above the mean rate across forest types; significance untested</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Study system: randomly selected plantation systems, i.e., Miyawaki system, mixed plantation (2 × 2 m spacing), and mixed plantation (3 × 3 m spacing). Measurements from rehabilitated mining sites were used to assess carbon sequestration potential and the feasibility of ecosystem rehabilitation, considering the time to carbon payback and the Carbon Neutral Mining Index (CNMI) for sustainable recovery. The biomass was measured using a destructive method; subsequently, total carbon was calculated by multiplying the biomass by the IPCC default coefficient of 0.475. - not clear how many plants, biomass per plant, what the method was, etc.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1684,17 +1643,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC6" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Using allometric equations, the estimate of  total above-ground and belowground biomass was 42.15 t dry matter ha-1 and for carbon, 18.74 t C ha-1. </t>
-        </is>
-      </c>
-      <c r="AD6" s="9" t="n"/>
-      <c r="AE6" s="9" t="inlineStr">
-        <is>
-          <t>Used allometric equations to estimate C stocks. Does a back-of-the-envelope calculation of C stocks in Miyawaki forests compared to other types of reforestation in the text, but doesn't do a meta-analysis. https://maps.app.goo.gl/BSL9kjsVGH55T7VA6</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1829,17 +1777,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC7" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Miyawaki forest reached total species richness of shrine forests. </t>
-        </is>
-      </c>
-      <c r="AD7" s="9" t="n"/>
-      <c r="AE7" s="9" t="inlineStr">
-        <is>
-          <t>Compared Miyawaki forest species counts to those in a shrine forest (not planted - remnant forest plots). No error bars/statistics</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1971,11 +1908,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>Plants show temporal variation in photosynthetic rate, transpiration, basal diameter, and height.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -2108,16 +2040,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>Soil elements and physicochemical variables (except % soil moisture) varied significantly over time within Miyawaki forest and among plots.</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>Comparison was made between a single Miyawaki forest plot and a single secondary forest plot. On university campus: https://maps.app.goo.gl/fSKpHtjk7kuWE4h77. Soil % organic C and % organic matter in Miyawaki forest tend to decline over time (17 years) and tend to be lower than secondary forests, but wrong statistical model was run (repeated measures treated as independent variables in ANOVA).</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2250,11 +2172,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC10" s="21" t="inlineStr">
-        <is>
-          <t>By year 6, individual density and %evergreen trees reached maxima of approximately 16000 individuals·ha⁻¹ and 90%, respectively. Individual density declined over time. By year 12, the relative biomass of evergreens was approximately 40–50%.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2388,11 +2305,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mini Forest student participants report high levels of civic participation and nature connectedness.  </t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -2526,17 +2438,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC12" s="11" t="inlineStr">
-        <is>
-          <t>Highest carbon stock and sequestration rate was calculated for the oldest Mini Forest.</t>
-        </is>
-      </c>
-      <c r="AD12" s="11" t="n"/>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pseudoreplicates within a forest plot were calculated via bootstrapping at 2000 iterations. </t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2670,16 +2571,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>The calculated carbon stock of selected 34 tree species ranged from 0.06 to 3.83 kg tree-1, while carbon dioxide equivalent (CO2e) ranged from 0.23 to 14.03 kg tree-1.</t>
-        </is>
-      </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>Compared to "an adjacent open natural tree stand"</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -2813,17 +2704,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC14" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Soil carbon concentration, respiration rate, microbial biomass were significantly higher in Mini Forests compared to nearby lawns. </t>
-        </is>
-      </c>
-      <c r="AD14" s="11" t="n"/>
-      <c r="AE14" t="inlineStr">
-        <is>
-          <t>The control areas were undisturbed soil covered with lawn and located at least three meters away from the microforests. Unclear the age of the lawns. Miyawaki forest plots were planted in 2021, 2022, 2023 - sampling occurred in 2024.</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -2904,7 +2784,7 @@
       </c>
       <c r="Q15" s="9" t="inlineStr">
         <is>
-          <t>Practitioners thoughts and feelings about Miyawaki forests (interviews and surveys)</t>
+          <t>Practitioners thoughts and feelings about Mini Forests (interviews and surveys)</t>
         </is>
       </c>
       <c r="R15" s="9" t="inlineStr">
@@ -2962,12 +2842,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC15" s="9" t="inlineStr">
-        <is>
-          <t>In urban areas, the most recommended Mini Forest locations are close to educational or health facilities. Half the interviewees believe that for Mini Forests to be accepted by the public, the method would need to be explained and well introduced. Almost all (11/12) interviewees considered costs to be an important constraint for applying Mini Forests; interviewees with experience planting Mini forests stated that it requires 3–4 times the budget of traditional tree planting.</t>
-        </is>
-      </c>
-      <c r="AD15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -3102,17 +2976,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC16" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Each planting day mobilized dozens of volunteers: most participants were not locals (e.g., underserved communities), but were already members of the local garden club. Mini Forests created potential for mutual learning between citizens and practitioners. </t>
-        </is>
-      </c>
-      <c r="AD16" s="9" t="n"/>
-      <c r="AE16" s="9" t="inlineStr">
-        <is>
-          <t>Enthographic study - found that most participants were not locals (e.g., underserved communities), but were already members of the local garden club</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3251,11 +3114,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>Mini Forests have clear Theory of Change that directs activity: staff and coordinators aim for transitions at policy and cultural (general public) level, while volunteering citizens focus on short-term aspects, such as creating more green space in their neighbourhood together with their community. Stakeholders identified four key factors driving the success of the Mini Forest programs: (1) starting and maintaining the Forest is a tangible activity with a visible result, (2) Mini Forests are connected to a local neighborhood, (3) it is a nationwide concept with critical mass, (4) external funding is key to the program implementation</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="13" t="inlineStr">
@@ -3390,17 +3248,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC18" s="13" t="inlineStr">
-        <is>
-          <t>Simulated deposition flux for NO2, Utilization factors for (a) Technological solutions and (b) Ecological solutions, (c) Sustainability index for Miyawaki plots with different managements and for traditional tree planting.</t>
-        </is>
-      </c>
-      <c r="AD18" s="13" t="n"/>
-      <c r="AE18" s="13" t="inlineStr">
-        <is>
-          <t>This is a very odd study where they just ran iTree for a Miyawaki forest with and without pruning. They also ran it for a "traditional" type of reforestation (i.e., slower growing trees? It's not described) and a tech approach to reducing atmospheric CO2 and NO2: selective catalytic reactor and monoethanolamine. (urban parameters used for models), although no study system described. To simulate the Miyawaki forest, they collected "remote sensing data and pre-processing, (2) Computation of vegetation indices, (3) Detection of tree species, (4) Populating tree inventories, and finally importing to i-Tree suite and simulation to calculate deposition flux. Focused on two megacities in India, New Delhi, and Chennai.</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -3481,7 +3328,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Projected distribution of plant canopy in existing Miyawaki forests</t>
+          <t>Projected distribution of plant canopy in existing Mini Forests</t>
         </is>
       </c>
       <c r="R19" s="13" t="inlineStr">
@@ -3533,13 +3380,6 @@
       <c r="AB19" s="13" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AC19" s="13" t="n"/>
-      <c r="AD19" s="13" t="n"/>
-      <c r="AE19" s="13" t="inlineStr">
-        <is>
-          <t>No study system was described. Used "urban forest" parameters in model</t>
         </is>
       </c>
     </row>
@@ -3676,9 +3516,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC20" s="14" t="n"/>
-      <c r="AD20" s="14" t="n"/>
-      <c r="AE20" s="14" t="n"/>
     </row>
     <row r="21" customFormat="1" s="14">
       <c r="A21" s="13" t="inlineStr">
@@ -4583,7 +4420,7 @@
       </c>
       <c r="Q29" s="13" t="inlineStr">
         <is>
-          <t>Extent of degradation of land slated for Miyawaki forest</t>
+          <t>Extent of degradation of land slated for Mini Forest</t>
         </is>
       </c>
       <c r="R29" s="13" t="inlineStr">
@@ -4609,13 +4446,6 @@
       <c r="Z29" s="13" t="n"/>
       <c r="AA29" s="13" t="n"/>
       <c r="AB29" s="13" t="n"/>
-      <c r="AC29" s="13" t="n"/>
-      <c r="AD29" s="13" t="n"/>
-      <c r="AE29" s="13" t="inlineStr">
-        <is>
-          <t>Peri-urban (forest outside of Hanzhong): https://maps.app.goo.gl/kPNjocS23UVyNgMQ8</t>
-        </is>
-      </c>
     </row>
     <row r="30" customFormat="1" s="14">
       <c r="A30" s="9" t="inlineStr">
@@ -4748,16 +4578,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC30" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">On average, across species, survival rate was 92% after 1 year, 87% after 3 years in Miyawaki forest vs. 72% in "conventional method" plot (no method was described). </t>
-        </is>
-      </c>
-      <c r="AE30" t="inlineStr">
-        <is>
-          <t>Only compared "survival rate" of plants between one Miyawaki plot and a "conventional method" plot. No description of "conventional method" that Miyawaki was compared to. No replicate plots or sample data reported., iron ore mines in rural area: https://maps.app.goo.gl/B6ArGFhQT4NMFKfa9</t>
-        </is>
-      </c>
     </row>
     <row r="31" customFormat="1" s="14">
       <c r="A31" s="9" t="inlineStr">
@@ -4890,17 +4710,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC31" s="9" t="inlineStr">
-        <is>
-          <t>Mortality rates were 15.84%, 22.98%, and 61% (site A) and 10.24%, 35.25%, and 84.29% (site B) for Miyawaki plots. Plots differ significantly in height of individual species.</t>
-        </is>
-      </c>
-      <c r="AD31" s="9" t="n"/>
-      <c r="AE31" s="9" t="inlineStr">
-        <is>
-          <t>For traditional methods: "Techniques involved planting along countour lines after forming gradoni or terraces by subsoiling, or along the maximum slope with subsoiling and holes." These sites are 15 years old, compared to the 10 year old Miyawaki forest plots!! Very little analysis was conducted. Statistical tests only on abundance (# plants) of individual species across plots, but it is very difficult to interpret. Plant density is higher in Miyawaki forests, but no statistical tests were conducted on plant height. Based on the graphics, there is no clear indication that diversity, plant growth rate is greater in MIyawaki forests. https://maps.app.goo.gl/tkfGdH1UTeDJfgAk8</t>
-        </is>
-      </c>
     </row>
     <row r="32" customFormat="1" s="14">
       <c r="A32" s="9" t="inlineStr">
@@ -5031,16 +4840,6 @@
       <c r="AB32" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AC32" t="inlineStr">
-        <is>
-          <t>85% of the trees of low-slope sites were higher than those of high-slope sites.</t>
-        </is>
-      </c>
-      <c r="AE32" t="inlineStr">
-        <is>
-          <t>Compared to a natural nearby beech wood. Overgrazed rural area: https://maps.app.goo.gl/SYcqJaBdSnQ3fRH19</t>
         </is>
       </c>
     </row>
@@ -5693,11 +5492,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC38" s="14" t="inlineStr">
-        <is>
-          <t>Average plant height, % cover, species richness per Miyawaki plot after a certain number of years (varies by plot). Stem count per species per plot.</t>
-        </is>
-      </c>
     </row>
     <row r="39" customFormat="1" s="14">
       <c r="A39" s="13" t="inlineStr">
@@ -5830,17 +5624,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC39" s="13" t="inlineStr">
-        <is>
-          <t>Survival rate per species at 6 months, 20 months in single Miyawaki forest plot</t>
-        </is>
-      </c>
-      <c r="AD39" s="13" t="n"/>
-      <c r="AE39" s="13" t="inlineStr">
-        <is>
-          <t>Just studied one Miyawaki forest plot. https://maps.app.goo.gl/dSPj7ymsRDEi5hrq9</t>
-        </is>
-      </c>
     </row>
     <row r="40" customFormat="1" s="14">
       <c r="A40" s="13" t="inlineStr">
@@ -5975,16 +5758,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC40" s="14" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AE40" s="14" t="inlineStr">
-        <is>
-          <t>Study conducted on two plots: one Miyawaki forest plot and one food forest plot. Reported higher establishment cost for Miyawaki vs. food forest. Also reported similar soil microbial populations across plots. No statistical tests run. https://maps.app.goo.gl/dSPj7ymsRDEi5hrq9</t>
-        </is>
-      </c>
     </row>
     <row r="41" customFormat="1" s="14">
       <c r="A41" s="13" t="inlineStr">
@@ -6119,11 +5892,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AE41" s="14" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/PoERdSJXFPNLfAFa9. Two plantation methods were evaluated: Miyawaki Plantation: Conducted on a 330 sq. meters plot, Conventional (control) Plantation: Conducted on a larger area of 3385 sq. meters.</t>
-        </is>
-      </c>
     </row>
     <row r="42" customFormat="1" s="14">
       <c r="A42" s="14" t="inlineStr">
@@ -6204,7 +5972,7 @@
       </c>
       <c r="Q42" s="14" t="inlineStr">
         <is>
-          <t>Modeled plant cover and thermal conditions over time, using policy documents, remote sensing data for the town, and literature on Miyawaki forests.</t>
+          <t>Modeled plant cover and thermal conditions over time, using policy documents, remote sensing data for the town, and literature on Mini Forests.</t>
         </is>
       </c>
       <c r="R42" s="14" t="inlineStr">
@@ -6251,11 +6019,6 @@
       <c r="AB42" s="14" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AE42" s="14" t="inlineStr">
-        <is>
-          <t>Uses "secondary data": the key data sources include: • Government reports and official documents related to the Upvan Scheme and urban forestry initiatives in Uttar Pradesh. • Satellite-based studies and open-access remote sensing literature reporting NDVI and LST trends for Lucknow. • Peer-reviewed academic articles on UHI, urban greening, and Miyawaki plantations in Indian and global contexts.</t>
         </is>
       </c>
     </row>
@@ -6467,7 +6230,7 @@
       </c>
       <c r="Q44" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interests in, Perception of, and opinions regarding the Miyawaki forest concept of the University of Agronomic Sciences and Veterinary Medicine of Bucharest (UASVM-B) students </t>
+          <t xml:space="preserve">Interests in, Perception of, and opinions regarding the Mini Forest concept of the University of Agronomic Sciences and Veterinary Medicine of Bucharest (UASVM-B) students </t>
         </is>
       </c>
       <c r="R44" s="14" t="inlineStr">
@@ -6646,8 +6409,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC45" s="13" t="n"/>
-      <c r="AD45" s="13" t="n"/>
     </row>
     <row r="46" customFormat="1" s="14">
       <c r="A46" s="13" t="inlineStr">
@@ -6782,13 +6543,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC46" s="13" t="n"/>
-      <c r="AD46" s="13" t="n"/>
-      <c r="AE46" s="16" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/XcRSDtTDz8kf1PSz7</t>
-        </is>
-      </c>
     </row>
     <row r="47" customFormat="1" s="14">
       <c r="A47" s="13" t="inlineStr">
@@ -6917,13 +6671,6 @@
       <c r="AB47" s="13" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AC47" s="13" t="n"/>
-      <c r="AD47" s="13" t="n"/>
-      <c r="AE47" s="16" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/gjyzkYCy96fvH4ir5</t>
         </is>
       </c>
     </row>
@@ -7032,8 +6779,6 @@
       <c r="Z48" s="13" t="n"/>
       <c r="AA48" s="13" t="n"/>
       <c r="AB48" s="13" t="n"/>
-      <c r="AC48" s="13" t="n"/>
-      <c r="AD48" s="13" t="n"/>
     </row>
     <row r="49" customFormat="1" s="14">
       <c r="A49" s="13" t="inlineStr">
@@ -7137,11 +6882,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="AE49" s="14" t="inlineStr">
-        <is>
-          <t>Online it says it is referreed, but I really don't think it is: https://repositorio.udd.cl/communities/0f16245b-c75b-43cf-86f1-4f986499804e</t>
-        </is>
-      </c>
     </row>
     <row r="50" customFormat="1" s="14">
       <c r="A50" s="13" t="inlineStr">
@@ -7280,11 +7020,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AE50" s="14" t="inlineStr">
-        <is>
-          <t>At the Carinthia University of Applied Sciences (CUAS): https://maps.app.goo.gl/qNBG9Nq2Xoz9nXcg7</t>
-        </is>
-      </c>
     </row>
     <row r="51" customFormat="1" s="14">
       <c r="A51" s="13" t="inlineStr">
@@ -7384,11 +7119,6 @@
         </is>
       </c>
       <c r="U51" s="26" t="n"/>
-      <c r="AE51" s="14" t="inlineStr">
-        <is>
-          <t>No study system was described. It's a review article</t>
-        </is>
-      </c>
     </row>
     <row r="52" customFormat="1" s="14">
       <c r="A52" s="14" t="inlineStr">
@@ -7591,11 +7321,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="AE53" s="14" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/4fT8cno477dGQrhC9</t>
-        </is>
-      </c>
     </row>
     <row r="54" customFormat="1" s="14">
       <c r="A54" s="14" t="inlineStr">
@@ -8651,17 +8376,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC63" s="13" t="inlineStr">
-        <is>
-          <t>Average plant height and biomass per species in single Miyawaki plot over time.</t>
-        </is>
-      </c>
-      <c r="AD63" s="13" t="n"/>
-      <c r="AE63" s="13" t="inlineStr">
-        <is>
-          <t>Single Miyawaki forest site measured. In a forest reserve after removing invasive plant: https://maps.app.goo.gl/fNnk95pobCFscitf7.</t>
-        </is>
-      </c>
     </row>
     <row r="64" customFormat="1" s="14">
       <c r="A64" s="13" t="inlineStr">
@@ -8796,11 +8510,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AE64" s="14" t="inlineStr">
-        <is>
-          <t>"The 20-cent area was divided into 4 equal plots 20 × 10 square metres each. Three plots were research plots R1, R2 and R3. The last quarter served as control.". Unclear how control plots were handled (i.e., if soil was amended in same way as Miyawaki plots), but authors say that: mycorrhizal inoculum and mulch was only applied to "experimental plots", and that the control plots had "normal spacing". Samples collected after 29 months of growth. Only compared plant biomass and growth rate to "control" plots - didn't calculate C sequestration for controls.  https://maps.app.goo.gl/FhkfnqsPzCvunKVE9.</t>
-        </is>
-      </c>
     </row>
     <row r="65" customFormat="1" s="14">
       <c r="A65" s="13" t="inlineStr">
@@ -8935,11 +8644,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AE65" s="17" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/57QUpkKnZDJgoTxSA</t>
-        </is>
-      </c>
     </row>
     <row r="66" customFormat="1" s="14">
       <c r="A66" s="14" t="inlineStr">
@@ -9067,11 +8771,6 @@
       <c r="AB66" s="14" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AE66" s="14" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/PF5RZDBtPebmvXTu8</t>
         </is>
       </c>
     </row>
@@ -9287,8 +8986,6 @@
       <c r="Z68" s="13" t="n"/>
       <c r="AA68" s="13" t="n"/>
       <c r="AB68" s="13" t="n"/>
-      <c r="AC68" s="13" t="n"/>
-      <c r="AD68" s="13" t="n"/>
     </row>
     <row r="69" customFormat="1" s="14">
       <c r="A69" s="13" t="inlineStr">
@@ -9421,12 +9118,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC69" s="13" t="inlineStr">
-        <is>
-          <t>Average plant height per species over time in single Miyawaki plot over time.</t>
-        </is>
-      </c>
-      <c r="AD69" s="13" t="n"/>
     </row>
     <row r="70" customFormat="1" s="14">
       <c r="A70" s="13" t="inlineStr">
@@ -9537,13 +9228,6 @@
       <c r="Z70" s="13" t="n"/>
       <c r="AA70" s="13" t="n"/>
       <c r="AB70" s="13" t="n"/>
-      <c r="AC70" s="13" t="n"/>
-      <c r="AD70" s="13" t="n"/>
-      <c r="AE70" s="13" t="inlineStr">
-        <is>
-          <t>Reports amounts of carbon sequestered annually by Miyawaki forests, but doesn't describe any of the science: no study system, no methods, etc. The figure caption reads, "Calculated based on data from NSI". No study system is described</t>
-        </is>
-      </c>
     </row>
     <row r="71" customFormat="1" s="14">
       <c r="A71" s="13" t="inlineStr">
@@ -9786,17 +9470,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC72" s="13" t="inlineStr">
-        <is>
-          <t>% canopy closure, % class cover over time for two different Miyawaki forest plots compared to nearby sites. Stem counts of living and dead plants in each Miyawaki plot after 25-59 months (depending on plot).</t>
-        </is>
-      </c>
-      <c r="AD72" s="13" t="n"/>
-      <c r="AE72" s="14" t="inlineStr">
-        <is>
-          <t>There are replicate Miyawaki forest plots, but no replicated control or "traditional method" plots. Compared plant diversity and density of each species (count) to a previously published study of a nearby natural forest (national park)</t>
-        </is>
-      </c>
     </row>
     <row r="73" customFormat="1" s="14">
       <c r="A73" s="13" t="inlineStr">
@@ -9929,17 +9602,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC73" s="13" t="inlineStr">
-        <is>
-          <t>Average plant height per species within Miyawaki forest and "traditional" planting (lower density) plot</t>
-        </is>
-      </c>
-      <c r="AD73" s="13" t="n"/>
-      <c r="AE73" s="14" t="inlineStr">
-        <is>
-          <t>In Nairobi: https://maps.app.goo.gl/FRho9i2iWnS5pZK78. Replicate individuals of a plant species were measured within a single Miyawaki plot and a single "traditional planting method" plot. This is the extent of the methods description: "traditional planting method with a spacing of 1 m2 between the seedlings". No statistics were run, but there are error bars on the graph - I assume these are for different individuals of the same species in the Miyawaki forest vs. traditional planting plot</t>
-        </is>
-      </c>
     </row>
     <row r="74" customFormat="1" s="14">
       <c r="A74" s="13" t="inlineStr">
@@ -10072,16 +9734,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC74" s="14" t="inlineStr">
-        <is>
-          <t>Average height, % growth of plant species in the first 3 years.</t>
-        </is>
-      </c>
-      <c r="AE74" s="17" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/xcc3kcQEeaJVaH6m7</t>
-        </is>
-      </c>
     </row>
     <row r="75" customFormat="1" s="14">
       <c r="A75" s="13" t="inlineStr">
@@ -10216,17 +9868,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC75" s="13" t="inlineStr">
-        <is>
-          <t>Average plant height, biomass, number of leaves, number of branches per species. Richness of insects, mushroom-forming fungi across three Miyawaki forests.</t>
-        </is>
-      </c>
-      <c r="AD75" s="13" t="n"/>
-      <c r="AE75" s="14" t="inlineStr">
-        <is>
-          <t>I can't find any real comparison of growth rates. No statistics. Also, no information about the "control" site is given: age of plants, etc. https://maps.app.goo.gl/ZvjmR6NJrknGbSBL9</t>
-        </is>
-      </c>
     </row>
     <row r="76" customFormat="1" s="14">
       <c r="A76" s="13" t="inlineStr">
@@ -10361,13 +10002,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC76" s="13" t="n"/>
-      <c r="AD76" s="13" t="n"/>
-      <c r="AE76" s="16" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/AkXuDLsm6QJBVqRG6</t>
-        </is>
-      </c>
     </row>
     <row r="77" customFormat="1" s="14">
       <c r="A77" s="13" t="inlineStr">
@@ -10502,13 +10136,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AC77" s="13" t="n"/>
-      <c r="AD77" s="13" t="n"/>
-      <c r="AE77" s="16" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/AkXuDLsm6QJBVqRG6</t>
-        </is>
-      </c>
     </row>
     <row r="78" customFormat="1" s="14">
       <c r="A78" s="14" t="inlineStr">
@@ -11049,11 +10676,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AE81" s="14" t="inlineStr">
-        <is>
-          <t>This study appeared to compare soil microbial abundances to a set of forests, and to compare animal diversity to "reference plots" matched to the two Miyawaki forests, but no details were provided on what those plots were.</t>
-        </is>
-      </c>
     </row>
     <row r="82" customFormat="1" s="14">
       <c r="A82" s="14" t="inlineStr">
@@ -11134,7 +10756,7 @@
       </c>
       <c r="Q82" s="14" t="inlineStr">
         <is>
-          <t>Animal biodiversity, plant biodiversity, plant carbon sequestration, tree growth rate, tree biomass, air temperature, soil temperature, precipitation experienced by each Miyawaki forest</t>
+          <t>Animal biodiversity, plant biodiversity, plant carbon sequestration, tree growth rate, tree biomass, air temperature, soil temperature, precipitation experienced by each Mini Forest</t>
         </is>
       </c>
       <c r="R82" s="14" t="inlineStr">
@@ -11186,16 +10808,6 @@
       <c r="AB82" s="14" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AC82" s="14" t="inlineStr">
-        <is>
-          <t>Air and soil temperatures (compared to nearby lawns, although method of matching is unclear. No information about lawns is included).</t>
-        </is>
-      </c>
-      <c r="AE82" s="14" t="inlineStr">
-        <is>
-          <t>Soil and air temperatures of the adjacent ornamental lawn and street were also measured</t>
         </is>
       </c>
     </row>
@@ -11413,7 +11025,7 @@
       </c>
       <c r="Q84" s="14" t="inlineStr">
         <is>
-          <t>Expectations, communication and  perceived cultural/ecological services of plantings, Miyawaki forest costs</t>
+          <t>Expectations, communication and  perceived cultural/ecological services of plantings, Mini Forest costs</t>
         </is>
       </c>
       <c r="R84" s="14" t="inlineStr">
@@ -11465,11 +11077,6 @@
       <c r="AB84" s="14" t="inlineStr">
         <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="AE84" s="14" t="inlineStr">
-        <is>
-          <t>This is a survey of people who have participated in Miyawaki forest plantings in France</t>
         </is>
       </c>
     </row>
@@ -13370,8 +12977,6 @@
       <c r="Z101" s="18" t="n"/>
       <c r="AA101" s="18" t="n"/>
       <c r="AB101" s="18" t="n"/>
-      <c r="AC101" s="18" t="n"/>
-      <c r="AD101" s="18" t="n"/>
     </row>
     <row r="102" customFormat="1" s="14">
       <c r="A102" s="14" t="inlineStr">
@@ -13696,11 +13301,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AE104" s="14" t="inlineStr">
-        <is>
-          <t>Results calculated for a hypothetical tiny forest, using data on tree species from three tiny firests in the Netherlands</t>
-        </is>
-      </c>
     </row>
     <row r="105" customFormat="1" s="14">
       <c r="A105" s="14" t="inlineStr">
@@ -13876,7 +13476,7 @@
       </c>
       <c r="Q106" s="14" t="inlineStr">
         <is>
-          <t>Tree crown detection and localization, tree biomass, tree growth rate, and wood volume, and terrain of Miyawaki forest</t>
+          <t>Tree crown detection and localization, tree biomass, tree growth rate, and wood volume, and terrain of Mini Forest</t>
         </is>
       </c>
       <c r="R106" s="14" t="inlineStr">
@@ -14217,14 +13817,6 @@
       <c r="U109" s="26" t="n"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF46" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF47" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF65" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF74" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF76" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AF77" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>